<commit_message>
Added some checks so that it doesn't crash if a book on the site isn't formated as expected
</commit_message>
<xml_diff>
--- a/outPutFile.xlsx
+++ b/outPutFile.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="3pages of books" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="10pages of books" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B72"/>
+  <dimension ref="A1:B240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1220,6 +1220,1882 @@
         </is>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" t="inlineStr"/>
+      <c r="B73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Page: 4</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr"/>
+      <c r="B75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>The Nameless City (The Nameless City #1)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>£38.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>The Murder That Never Was (Forensic Instincts #5)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>£54.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>The Most Perfect Thing: Inside (and Outside) a Bird's Egg</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>£42.96</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>The Mindfulness and Acceptance Workbook for Anxiety: A Guide to Breaking Free from Anxiety, Phobias, and Worry Using Acceptance and Commitment Therapy</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>£23.89</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>The Life-Changing Magic of Tidying Up: The Japanese Art of Decluttering and Organizing</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>£16.77</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>The Inefficiency Assassin: Time Management Tactics for Working Smarter, Not Longer</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>£20.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>The Gutsy Girl: Escapades for Your Life of Epic Adventure</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>£37.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>The Electric Pencil: Drawings from Inside State Hospital No. 3</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>£56.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>The Death of Humanity: and the Case for Life</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>£58.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>The Bulletproof Diet: Lose up to a Pound a Day, Reclaim Energy and Focus, Upgrade Your Life</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>£49.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>The Art Forger</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>£40.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>The Age of Genius: The Seventeenth Century and the Birth of the Modern Mind</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>£19.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>The Activist's Tao Te Ching: Ancient Advice for a Modern Revolution</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>£32.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Spark Joy: An Illustrated Master Class on the Art of Organizing and Tidying Up</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>£41.83</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Soul Reader</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>£39.58</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>£39.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Saga, Volume 6 (Saga (Collected Editions) #6)</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>£25.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Saga, Volume 5 (Saga (Collected Editions) #5)</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>£51.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Reskilling America: Learning to Labor in the Twenty-First Century</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>£19.83</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Rat Queens, Vol. 3: Demons (Rat Queens (Collected Editions) #11-15)</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>£50.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr"/>
+      <c r="B97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Page: 5</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr"/>
+      <c r="B99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Princess Jellyfish 2-in-1 Omnibus, Vol. 01 (Princess Jellyfish 2-in-1 Omnibus #1)</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>£13.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Princess Between Worlds (Wide-Awake Princess #5)</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>£13.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Pop Gun War, Volume 1: Gift</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>£18.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Political Suicide: Missteps, Peccadilloes, Bad Calls, Backroom Hijinx, Sordid Pasts, Rotten Breaks, and Just Plain Dumb Mistakes in the Annals of American Politics</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>£36.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Patience</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>£10.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Outcast, Vol. 1: A Darkness Surrounds Him (Outcast #1)</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>£15.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>orange: The Complete Collection 1 (orange: The Complete Collection #1)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>£48.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Online Marketing for Busy Authors: A Step-By-Step Guide</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>£46.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>On a Midnight Clear</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>£14.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Obsidian (Lux #1)</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>£14.86</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>My Paris Kitchen: Recipes and Stories</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>£33.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Masks and Shadows</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>£56.40</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Mama Tried: Traditional Italian Cooking for the Screwed, Crude, Vegan, and Tattooed</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>£14.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Lumberjanes, Vol. 2: Friendship to the Max (Lumberjanes #5-8)</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>£46.91</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Lumberjanes, Vol. 1: Beware the Kitten Holy (Lumberjanes #1-4)</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>£45.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Lumberjanes Vol. 3: A Terrible Plan (Lumberjanes #9-12)</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>£19.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Layered: Baking, Building, and Styling Spectacular Cakes</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>£40.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Judo: Seven Steps to Black Belt (an Introductory Guide for Beginners)</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>£53.90</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Join</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>£35.67</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>In the Country We Love: My Family Divided</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>£22.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr"/>
+      <c r="B121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Page: 6</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr"/>
+      <c r="B123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Immunity: How Elie Metchnikoff Changed the Course of Modern Medicine</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>£57.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>I Hate Fairyland, Vol. 1: Madly Ever After (I Hate Fairyland (Compilations) #1-5)</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>£29.17</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>I am a Hero Omnibus Volume 1</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>£54.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>How to Be Miserable: 40 Strategies You Already Use</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>£46.03</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Her Backup Boyfriend (The Sorensen Family #1)</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>£33.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Giant Days, Vol. 2 (Giant Days #5-8)</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>£22.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Forever and Forever: The Courtship of Henry Longfellow and Fanny Appleton</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>£29.69</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>First and First (Five Boroughs #3)</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>£15.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Fifty Shades Darker (Fifty Shades #2)</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>£21.96</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Everydata: The Misinformation Hidden in the Little Data You Consume Every Day</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>£54.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Don't Be a Jerk: And Other Practical Advice from Dogen, Japan's Greatest Zen Master</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>£37.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Danganronpa Volume 1</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>£51.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Crown of Midnight (Throne of Glass #2)</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>£43.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Codename Baboushka, Volume 1: The Conclave of Death</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>£36.72</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Camp Midnight</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>£17.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Call the Nurse: True Stories of a Country Nurse on a Scottish Isle</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>£29.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Burning</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>£28.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Bossypants</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>£49.46</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Bitch Planet, Vol. 1: Extraordinary Machine (Bitch Planet (Collected Editions))</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>£37.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Avatar: The Last Airbender: Smoke and Shadow, Part 3 (Smoke and Shadow #3)</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>£28.09</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr"/>
+      <c r="B145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Page: 7</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr"/>
+      <c r="B147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Algorithms to Live By: The Computer Science of Human Decisions</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>£30.81</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>A World of Flavor: Your Gluten Free Passport</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>£42.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>A Piece of Sky, a Grain of Rice: A Memoir in Four Meditations</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>£56.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>A Murder in Time</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>£16.64</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>A Flight of Arrows (The Pathfinders #2)</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>£55.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>A Fierce and Subtle Poison</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>£28.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>A Court of Thorns and Roses (A Court of Thorns and Roses #1)</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>£52.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>(Un)Qualified: How God Uses Broken People to Do Big Things</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>£54.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>You Are What You Love: The Spiritual Power of Habit</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>£21.87</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>William Shakespeare's Star Wars: Verily, A New Hope (William Shakespeare's Star Wars #4)</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>£43.30</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Tuesday Nights in 1980</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>£21.04</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Tracing Numbers on a Train</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>£41.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Throne of Glass (Throne of Glass #1)</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>£35.07</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Thomas Jefferson and the Tripoli Pirates: The Forgotten War That Changed American History</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>£59.64</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Thirteen Reasons Why</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>£52.72</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>The White Cat and the Monk: A Retelling of the Poem “Pangur Bán”</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>£58.08</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>The Wedding Dress</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>£24.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>The Vacationers</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>£42.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>The Third Wave: An Entrepreneur’s Vision of the Future</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>£12.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>The Stranger</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>£17.44</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr"/>
+      <c r="B169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Page: 8</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr"/>
+      <c r="B171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>The Shadow Hero (The Shadow Hero)</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>£33.14</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>The Secret (The Secret #1)</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>£27.37</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>The Regional Office Is Under Attack!</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>£51.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>The Psychopath Test: A Journey Through the Madness Industry</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>£36.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>The Project</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>£10.65</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>The Power of Now: A Guide to Spiritual Enlightenment</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>£43.54</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>The Omnivore's Dilemma: A Natural History of Four Meals</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>£38.21</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>The Nerdy Nummies Cookbook: Sweet Treats for the Geek in All of Us</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>£37.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>The Murder of Roger Ackroyd (Hercule Poirot #4)</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>£44.10</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>The Mistake (Off-Campus #2)</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>£43.29</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>The Matchmaker's Playbook (Wingmen Inc. #1)</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>£55.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>The Love and Lemons Cookbook: An Apple-to-Zucchini Celebration of Impromptu Cooking</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>£37.60</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>The Long Shadow of Small Ghosts: Murder and Memory in an American City</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>£10.97</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>The Kite Runner</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>£41.82</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>The House by the Lake</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>£36.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>The Glittering Court (The Glittering Court #1)</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>£44.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>The Girl on the Train</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>£55.02</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>The Genius of Birds</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>£17.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>The Emerald Mystery</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>£23.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>The Cookies &amp; Cups Cookbook: 125+ sweet &amp; savory recipes reminding you to Always Eat Dessert First</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>£41.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr"/>
+      <c r="B193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Page: 9</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr"/>
+      <c r="B195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>The Bridge to Consciousness: I'm Writing the Bridge Between Science and Our Old and New Beliefs.</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>£32.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>The Artist's Way: A Spiritual Path to Higher Creativity</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>£38.49</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>The Art of War</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>£33.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>The Argonauts</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>£10.93</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>The 10% Entrepreneur: Live Your Startup Dream Without Quitting Your Day Job</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>£27.55</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Suddenly in Love (Lake Haven #1)</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>£55.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Something More Than This</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>£16.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Soft Apocalypse</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>£26.12</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>So You've Been Publicly Shamed</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>£12.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Shoe Dog: A Memoir by the Creator of NIKE</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>£23.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Shobu Samurai, Project Aryoku (#3)</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>£29.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Secrets and Lace (Fatal Hearts #1)</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>£20.27</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Scarlett Epstein Hates It Here</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>£43.55</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Romero and Juliet: A Tragic Tale of Love and Zombies</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>£36.94</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Redeeming Love</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>£20.47</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Poses for Artists Volume 1 - Dynamic and Sitting Poses: An Essential Reference for Figure Drawing and the Human Form</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>£41.06</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Poems That Make Grown Women Cry</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>£14.19</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Nightingale, Sing</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>£38.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Night Sky with Exit Wounds</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>£41.05</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Mrs. Houdini</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>£30.25</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr"/>
+      <c r="B217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Page: 10</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr"/>
+      <c r="B219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Modern Romance</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>£28.26</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Miss Peregrine’s Home for Peculiar Children (Miss Peregrine’s Peculiar Children #1)</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>£10.76</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Louisa: The Extraordinary Life of Mrs. Adams</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>£16.85</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Little Red</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>£13.47</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Library of Souls (Miss Peregrine’s Peculiar Children #3)</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>£48.56</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Large Print Heart of the Pride</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>£19.15</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>I Had a Nice Time And Other Lies...: How to find love &amp; sh*t like that</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>£57.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Hollow City (Miss Peregrine’s Peculiar Children #2)</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>£42.98</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Grumbles</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>£22.16</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Full Moon over Noah’s Ark: An Odyssey to Mount Ararat and Beyond</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>£49.43</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Frostbite (Vampire Academy #2)</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>£29.99</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Follow You Home</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>£21.36</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>First Steps for New Christians (Print Edition)</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>£29.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Finders Keepers (Bill Hodges Trilogy #2)</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>£53.53</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Fables, Vol. 1: Legends in Exile (Fables #1)</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>£41.62</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Eureka Trivia 6.0</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>£54.59</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Drive: The Surprising Truth About What Motivates Us</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>£34.95</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Done Rubbed Out (Reightman &amp; Bailey #1)</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>£37.72</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Doing It Over (Most Likely To #1)</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>£35.61</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Deliciously Ella Every Day: Quick and Easy Recipes for Gluten-Free Snacks, Packed Lunches, and Simple Meals</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>£42.16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>